<commit_message>
Update review prompt and bell-curve config for 2026 round-table guidelines
</commit_message>
<xml_diff>
--- a/output/yearend_review_report.xlsx
+++ b/output/yearend_review_report.xlsx
@@ -49,12 +49,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -208,12 +208,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Bell Curve Chart'!$A$2:$A$4</f>
+              <f>'Bell Curve Chart'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Bell Curve Chart'!$B$2:$B$4</f>
+              <f>'Bell Curve Chart'!$B$2:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -232,12 +232,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Bell Curve Chart'!$A$2:$A$4</f>
+              <f>'Bell Curve Chart'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Bell Curve Chart'!$C$2:$C$4</f>
+              <f>'Bell Curve Chart'!$C$2:$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -900,11 +900,11 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Exceeds Expectations</t>
+          <t>Meets Expectations</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -940,250 +940,250 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Exceeds Expectations</t>
+          <t>Meets Expectations</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>E003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>E003</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Priya Nair</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>QA Lead</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n">
+      <c r="E4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Meets Expectations</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>E006</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Vikram Reddy</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Senior Developer</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E5" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Meets Expectations</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>E002</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Rahul Mehta</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Meets Expectations</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>E011</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Ananya Rao</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Team Lead</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="E7" s="2" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Meets Expectations</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>E012</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Rohit Sharma</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Junior Developer</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E8" s="2" t="n">
         <v>2.6</v>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>4.22</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>83.3</v>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Meets Expectations</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="n">
+      <c r="F8" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Needs Development</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>E006</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Vikram Reddy</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Senior Developer</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" s="3" t="n">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>E010</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Manoj Kumar</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="2" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="3" t="n">
-        <v>4.12</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>75</v>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Meets Expectations</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>E002</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Rahul Mehta</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Software Engineer</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>Meets Expectations</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>E011</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Ananya Rao</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Team Lead</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>3.79</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Meets Expectations</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>E012</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Rohit Sharma</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Junior Developer</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>3.66</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>Meets Expectations</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>E010</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Manoj Kumar</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Software Engineer</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" s="3" t="n">
+      <c r="G9" s="2" t="n">
         <v>3.62</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H9" s="2" t="n">
         <v>41.7</v>
       </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>Meets Expectations</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="n">
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Needs Development</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1220,11 +1220,11 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Meets Expectations</t>
+          <t>Unsatisfactory Performance</t>
         </is>
       </c>
       <c r="J10" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1260,11 +1260,11 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Meets Expectations</t>
+          <t>Unsatisfactory Performance</t>
         </is>
       </c>
       <c r="J11" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1300,11 +1300,11 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Below Expectations</t>
+          <t>Severe Compliance/Performance Issue</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -1340,11 +1340,11 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Below Expectations</t>
+          <t>Severe Compliance/Performance Issue</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3422,7 +3422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3466,16 +3466,16 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C2" s="5" t="n">
-        <v>20</v>
-      </c>
       <c r="D2" s="5" t="n">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -3485,34 +3485,72 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Below Expectations</t>
+          <t>Needs Development</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>16.7</v>
       </c>
       <c r="E4" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Unsatisfactory Performance</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Severe Compliance/Performance Issue</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="E6" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3527,7 +3565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3559,10 +3597,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>16.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -3572,22 +3610,48 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="C3" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Below Expectations</t>
+          <t>Needs Development</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C4" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Unsatisfactory Performance</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C5" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Severe Compliance/Performance Issue</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" t="n">
         <v>16.7</v>
       </c>
     </row>

</xml_diff>